<commit_message>
Località balneari aggiornate fino a 44°
</commit_message>
<xml_diff>
--- a/dataset/Localita_balneari_Nord_Adriatico.xlsx
+++ b/dataset/Localita_balneari_Nord_Adriatico.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10715930_polimi_it/Documents/NonparametricProject_2526/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leomarcellopoli/Documents/Nonparametric/Project/Non-parametric-Statistics-2025-2026/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{99A22634-AC7E-E441-B9E3-06766CCF2C39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9C40EB1-D1A3-F348-B589-856DCDC17EEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16200" yWindow="500" windowWidth="22200" windowHeight="19260" xr2:uid="{36792D4C-30BA-2241-B39E-83FA7B9759F6}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="11500" windowHeight="17140" xr2:uid="{36792D4C-30BA-2241-B39E-83FA7B9759F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="46">
   <si>
     <t>Lat</t>
   </si>
@@ -90,6 +90,90 @@
   </si>
   <si>
     <t>Veneto</t>
+  </si>
+  <si>
+    <t>Barricata (Porto Tolle)</t>
+  </si>
+  <si>
+    <t>Emilia-Romagna</t>
+  </si>
+  <si>
+    <t>Lido di Volano</t>
+  </si>
+  <si>
+    <t>Lido delle Nazioni</t>
+  </si>
+  <si>
+    <t>Lido di Pomposa</t>
+  </si>
+  <si>
+    <t>Lido degli Scacchi</t>
+  </si>
+  <si>
+    <t>Porto Garibaldi</t>
+  </si>
+  <si>
+    <t>Lido degli Estensi</t>
+  </si>
+  <si>
+    <t>Lido di Spina</t>
+  </si>
+  <si>
+    <t>Casal Borsetti</t>
+  </si>
+  <si>
+    <t>Marina Romea</t>
+  </si>
+  <si>
+    <t>Marina di Ravenna</t>
+  </si>
+  <si>
+    <t>Punta Marina</t>
+  </si>
+  <si>
+    <t>Lido Adriano</t>
+  </si>
+  <si>
+    <t>Lido di Dante</t>
+  </si>
+  <si>
+    <t>Lido di Classe</t>
+  </si>
+  <si>
+    <t>Lido di Savio</t>
+  </si>
+  <si>
+    <t>Milano Marittima</t>
+  </si>
+  <si>
+    <t>Cervia</t>
+  </si>
+  <si>
+    <t>Pinarella</t>
+  </si>
+  <si>
+    <t>Cesenatico</t>
+  </si>
+  <si>
+    <t>Gatteo a Mare</t>
+  </si>
+  <si>
+    <t>San Mauro Mare</t>
+  </si>
+  <si>
+    <t>Bellaria-Igea Marina</t>
+  </si>
+  <si>
+    <t>Rimini</t>
+  </si>
+  <si>
+    <t>Isola di Albarella</t>
+  </si>
+  <si>
+    <t>Porto Levante</t>
+  </si>
+  <si>
+    <t>Boccasette</t>
   </si>
 </sst>
 </file>
@@ -97,7 +181,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="0.00000000"/>
+    <numFmt numFmtId="164" formatCode="0.00000000"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -161,10 +245,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -501,7 +585,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD630E25-B43E-A540-B6BD-3DEDB25F318E}">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="46.1640625" defaultRowHeight="28" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="46.1640625" style="1"/>
@@ -692,45 +776,382 @@
       </c>
     </row>
     <row r="14" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
+      <c r="A14" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="5">
+        <v>45.0715</v>
+      </c>
+      <c r="D14" s="6">
+        <v>12.34</v>
+      </c>
     </row>
     <row r="15" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
+      <c r="A15" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="5">
+        <v>45.0488</v>
+      </c>
+      <c r="D15" s="6">
+        <v>12.364000000000001</v>
+      </c>
     </row>
     <row r="16" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-    </row>
-    <row r="17" spans="3:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-    </row>
-    <row r="18" spans="3:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-    </row>
-    <row r="19" spans="3:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C19" s="6"/>
-    </row>
-    <row r="20" spans="3:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C20" s="6"/>
-    </row>
-    <row r="21" spans="3:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C21" s="6"/>
-    </row>
-    <row r="22" spans="3:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C22" s="6"/>
-    </row>
-    <row r="23" spans="3:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C23" s="6"/>
-    </row>
-    <row r="24" spans="3:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C24" s="6"/>
-    </row>
-    <row r="25" spans="3:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C25" s="6"/>
+      <c r="A16" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="5">
+        <v>45.027799999999999</v>
+      </c>
+      <c r="D16" s="6">
+        <v>12.423299999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="5">
+        <v>44.854399999999998</v>
+      </c>
+      <c r="D17" s="6">
+        <v>12.471</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="5">
+        <v>44.8033</v>
+      </c>
+      <c r="D18" s="6">
+        <v>12.265599999999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="5">
+        <v>44.746200000000002</v>
+      </c>
+      <c r="D19" s="6">
+        <v>12.2454</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="5">
+        <v>44.718899999999998</v>
+      </c>
+      <c r="D20" s="6">
+        <v>12.2385</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" s="5">
+        <v>44.710900000000002</v>
+      </c>
+      <c r="D21" s="6">
+        <v>12.238300000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="5">
+        <v>44.678100000000001</v>
+      </c>
+      <c r="D22" s="6">
+        <v>12.239599999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23" s="5">
+        <v>44.660800000000002</v>
+      </c>
+      <c r="D23" s="6">
+        <v>12.244400000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C24" s="5">
+        <v>44.644399999999997</v>
+      </c>
+      <c r="D24" s="6">
+        <v>12.2464</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" s="5">
+        <v>44.553100000000001</v>
+      </c>
+      <c r="D25" s="6">
+        <v>12.28</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26" s="5">
+        <v>44.518500000000003</v>
+      </c>
+      <c r="D26" s="6">
+        <v>12.2698</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27" s="5">
+        <v>44.485599999999998</v>
+      </c>
+      <c r="D27" s="6">
+        <v>12.282299999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="5">
+        <v>44.442</v>
+      </c>
+      <c r="D28" s="6">
+        <v>12.2956</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" s="5">
+        <v>44.411700000000003</v>
+      </c>
+      <c r="D29" s="6">
+        <v>12.3109</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C30" s="5">
+        <v>44.386099999999999</v>
+      </c>
+      <c r="D30" s="6">
+        <v>12.3162</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C31" s="5">
+        <v>44.325200000000002</v>
+      </c>
+      <c r="D31" s="6">
+        <v>12.335000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C32" s="5">
+        <v>44.304400000000001</v>
+      </c>
+      <c r="D32" s="6">
+        <v>12.343500000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C33" s="5">
+        <v>44.2804</v>
+      </c>
+      <c r="D33" s="6">
+        <v>12.349299999999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C34" s="5">
+        <v>44.261099999999999</v>
+      </c>
+      <c r="D34" s="6">
+        <v>12.3453</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C35" s="5">
+        <v>44.242899999999999</v>
+      </c>
+      <c r="D35" s="6">
+        <v>12.3672</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C36" s="5">
+        <v>44.1995</v>
+      </c>
+      <c r="D36" s="6">
+        <v>12.401199999999999</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C37" s="5">
+        <v>44.170999999999999</v>
+      </c>
+      <c r="D37" s="6">
+        <v>12.4381</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C38" s="5">
+        <v>44.163600000000002</v>
+      </c>
+      <c r="D38" s="6">
+        <v>12.4452</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C39" s="5">
+        <v>44.143599999999999</v>
+      </c>
+      <c r="D39" s="6">
+        <v>12.466799999999999</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C40" s="5">
+        <v>44.056600000000003</v>
+      </c>
+      <c r="D40" s="6">
+        <v>12.571300000000001</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>